<commit_message>
style(viewer): minimal table design with header underline, borderless cells, and tuned column widths
</commit_message>
<xml_diff>
--- a/docs/examples/demonstration-charts.xlsx
+++ b/docs/examples/demonstration-charts.xlsx
@@ -179,7 +179,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -188,18 +188,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -207,14 +208,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1540,9 +1541,10 @@
   <dimension ref="B2:D16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="57.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="21" x14ac:dyDescent="0.4">
@@ -1661,8 +1663,11 @@
   <dimension ref="B2:E17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="48.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="21" x14ac:dyDescent="0.4">

</xml_diff>